<commit_message>
Update completed Colab results for all three final seeds
</commit_message>
<xml_diff>
--- a/submissions/2A202603012_BuiQuangVinh/results.xlsx
+++ b/submissions/2A202603012_BuiQuangVinh/results.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backbones" sheetId="1" r:id="R44b92772e7be48a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Training" sheetId="2" r:id="R2d78d9618d7b4c4d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inference" sheetId="3" r:id="R4e5ed3131d1a4d63"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Final" sheetId="4" r:id="R5703aeb31bd54df2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PerClass" sheetId="5" r:id="R8df61feb0d694861"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Latency" sheetId="6" r:id="Rcefdf49502c14179"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="7" r:id="Ra50bdcc1580840ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backbones" sheetId="1" r:id="R62ff27b4647a4282"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Training" sheetId="2" r:id="Ra20933375a5449da"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inference" sheetId="3" r:id="R3ef865acec874f15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Final" sheetId="4" r:id="R88f1534d7eeb4b54"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PerClass" sheetId="5" r:id="R3f19630c68944447"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Latency" sheetId="6" r:id="R47af4c76e9c945ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="7" r:id="R97ebadb82ce84fe1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -91,7 +91,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="27">
+  <x:cellXfs count="32">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -167,6 +167,24 @@
     <x:xf numFmtId="204" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="202" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="204" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -240,6 +258,23 @@
     </x:indexedColors>
   </x:colors>
 </x:styleSheet>
+</file>
+
+<file path=xl/featurePropertyBag/featurePropertyBag.xml><?xml version="1.0" encoding="utf-8"?>
+<xfpb:FeaturePropertyBags xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag">
+  <xfpb:bag type="Checkbox"/>
+  <xfpb:bag type="XFControls">
+    <xfpb:bagId k="CellControl">0</xfpb:bagId>
+  </xfpb:bag>
+  <xfpb:bag type="XFComplement">
+    <xfpb:bagId k="XFControls">1</xfpb:bagId>
+  </xfpb:bag>
+  <xfpb:bag type="XFComplements" extRef="XFComplementsMapperExtRef">
+    <xfpb:a k="MappedFeaturePropertyBags">
+      <xfpb:bagId>2</xfpb:bagId>
+    </xfpb:a>
+  </xfpb:bag>
+</xfpb:FeaturePropertyBags>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1717,12 +1752,20 @@
       <x:c r="B7" s="21" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="C7" s="22"/>
-      <x:c r="D7" s="22"/>
-      <x:c r="E7" s="22"/>
-      <x:c r="F7" s="22"/>
+      <x:c r="C7" s="22" t="n">
+        <x:v>0.976959752451448</x:v>
+      </x:c>
+      <x:c r="D7" s="22" t="n">
+        <x:v>0.9793963117774231</x:v>
+      </x:c>
+      <x:c r="E7" s="22" t="n">
+        <x:v>0.9828913601368692</x:v>
+      </x:c>
+      <x:c r="F7" s="22" t="n">
+        <x:v>0.13894177577701738</x:v>
+      </x:c>
       <x:c r="G7" s="7" t="str">
-        <x:v>Chưa có artifact; không đưa vào mean/std</x:v>
+        <x:v>Đã chạy test; 3.507 ảnh</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2012,22 +2055,22 @@
         <x:v>226</x:v>
       </x:c>
       <x:c r="C11" s="22" t="n">
-        <x:v>0.9818580047937846</x:v>
+        <x:v>0.9775349661588194</x:v>
       </x:c>
       <x:c r="D11" s="22" t="n">
-        <x:v>0.9557522123893806</x:v>
+        <x:v>0.9587020648967552</x:v>
       </x:c>
       <x:c r="E11" s="22" t="n">
-        <x:v>0.9686092342342343</x:v>
+        <x:v>0.9679863483217143</x:v>
       </x:c>
       <x:c r="F11" s="6" t="str">
         <x:v>F01</x:v>
       </x:c>
       <x:c r="G11" s="21" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="H11" s="23" t="n">
-        <x:v>0.00019907285506370954</x:v>
+        <x:v>0.001088014513165879</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="24" customHeight="1">
@@ -2038,22 +2081,22 @@
         <x:v>213</x:v>
       </x:c>
       <x:c r="C12" s="22" t="n">
-        <x:v>0.9952153110047847</x:v>
+        <x:v>0.9936356041619199</x:v>
       </x:c>
       <x:c r="D12" s="22" t="n">
         <x:v>0.9765258215962441</x:v>
       </x:c>
       <x:c r="E12" s="22" t="n">
-        <x:v>0.985781990521327</x:v>
+        <x:v>0.9850051725618933</x:v>
       </x:c>
       <x:c r="F12" s="6" t="str">
         <x:v>F01</x:v>
       </x:c>
       <x:c r="G12" s="21" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="H12" s="23" t="n">
-        <x:v>0</x:v>
+        <x:v>0.0013454881739710242</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="24" customHeight="1">
@@ -2064,22 +2107,22 @@
         <x:v>207</x:v>
       </x:c>
       <x:c r="C13" s="22" t="n">
-        <x:v>0.9717197338851433</x:v>
+        <x:v>0.9795283662794159</x:v>
       </x:c>
       <x:c r="D13" s="22" t="n">
-        <x:v>0.9951690821256038</x:v>
+        <x:v>0.9935587761674718</x:v>
       </x:c>
       <x:c r="E13" s="22" t="n">
-        <x:v>0.9832991569833675</x:v>
+        <x:v>0.986444797149525</x:v>
       </x:c>
       <x:c r="F13" s="6" t="str">
         <x:v>F01</x:v>
       </x:c>
       <x:c r="G13" s="21" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="H13" s="23" t="n">
-        <x:v>0.0033188424908732698</x:v>
+        <x:v>0.005932327865555321</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="24" customHeight="1">
@@ -2093,19 +2136,19 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D14" s="22" t="n">
-        <x:v>0.9780487804878049</x:v>
+        <x:v>0.9788617886178862</x:v>
       </x:c>
       <x:c r="E14" s="22" t="n">
-        <x:v>0.9888887537402389</x:v>
+        <x:v>0.989308430243903</x:v>
       </x:c>
       <x:c r="F14" s="6" t="str">
         <x:v>F01</x:v>
       </x:c>
       <x:c r="G14" s="21" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="H14" s="23" t="n">
-        <x:v>0.005289496562990819</x:v>
+        <x:v>0.0038102194225699544</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="24" customHeight="1">
@@ -2116,22 +2159,22 @@
         <x:v>213</x:v>
       </x:c>
       <x:c r="C15" s="22" t="n">
-        <x:v>0.9587155963302753</x:v>
+        <x:v>0.9530450761783301</x:v>
       </x:c>
       <x:c r="D15" s="22" t="n">
-        <x:v>0.9812206572769953</x:v>
+        <x:v>0.9827856025039123</x:v>
       </x:c>
       <x:c r="E15" s="22" t="n">
-        <x:v>0.9698375870069604</x:v>
+        <x:v>0.9676593087691664</x:v>
       </x:c>
       <x:c r="F15" s="6" t="str">
         <x:v>F01</x:v>
       </x:c>
       <x:c r="G15" s="21" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="H15" s="23" t="n">
-        <x:v>0</x:v>
+        <x:v>0.0037728885808810705</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="24" customHeight="1">
@@ -2142,22 +2185,22 @@
         <x:v>202</x:v>
       </x:c>
       <x:c r="C16" s="22" t="n">
-        <x:v>0.9851226576230908</x:v>
+        <x:v>0.9883897243714007</x:v>
       </x:c>
       <x:c r="D16" s="22" t="n">
-        <x:v>0.9801980198019802</x:v>
+        <x:v>0.9768976897689768</x:v>
       </x:c>
       <x:c r="E16" s="22" t="n">
-        <x:v>0.9826298451402358</x:v>
+        <x:v>0.9825719435437829</x:v>
       </x:c>
       <x:c r="F16" s="6" t="str">
         <x:v>F01</x:v>
       </x:c>
       <x:c r="G16" s="21" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="H16" s="23" t="n">
-        <x:v>0.00012191120884964967</x:v>
+        <x:v>0.00013224581670873544</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="24" customHeight="1">
@@ -2168,22 +2211,22 @@
         <x:v>215</x:v>
       </x:c>
       <x:c r="C17" s="22" t="n">
-        <x:v>0.9906540015285512</x:v>
+        <x:v>0.9891397047227378</x:v>
       </x:c>
       <x:c r="D17" s="22" t="n">
-        <x:v>0.9860465116279069</x:v>
+        <x:v>0.9875968992248062</x:v>
       </x:c>
       <x:c r="E17" s="22" t="n">
-        <x:v>0.9883394914149097</x:v>
+        <x:v>0.9883593515851912</x:v>
       </x:c>
       <x:c r="F17" s="6" t="str">
         <x:v>F01</x:v>
       </x:c>
       <x:c r="G17" s="21" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="H17" s="23" t="n">
-        <x:v>0.003334974386383038</x:v>
+        <x:v>0.002358433878234937</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="24" customHeight="1">
@@ -2194,22 +2237,22 @@
         <x:v>204</x:v>
       </x:c>
       <x:c r="C18" s="22" t="n">
-        <x:v>0.9797974644797592</x:v>
+        <x:v>0.9781141345689978</x:v>
       </x:c>
       <x:c r="D18" s="22" t="n">
-        <x:v>0.9509803921568627</x:v>
+        <x:v>0.949346405228758</x:v>
       </x:c>
       <x:c r="E18" s="22" t="n">
-        <x:v>0.9651677258466737</x:v>
+        <x:v>0.9635114855561572</x:v>
       </x:c>
       <x:c r="F18" s="6" t="str">
         <x:v>F01</x:v>
       </x:c>
       <x:c r="G18" s="21" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="H18" s="23" t="n">
-        <x:v>0.003640482181316009</x:v>
+        <x:v>0.003854341831756702</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="24" customHeight="1">
@@ -2220,22 +2263,22 @@
         <x:v>1822</x:v>
       </x:c>
       <x:c r="C19" s="22" t="n">
-        <x:v>0.9839199818861897</x:v>
+        <x:v>0.9841825912374343</x:v>
       </x:c>
       <x:c r="D19" s="22" t="n">
-        <x:v>0.9906695938529089</x:v>
+        <x:v>0.9903036955726309</x:v>
       </x:c>
       <x:c r="E19" s="22" t="n">
-        <x:v>0.987283086973139</x:v>
+        <x:v>0.987233345508327</x:v>
       </x:c>
       <x:c r="F19" s="6" t="str">
         <x:v>F01</x:v>
       </x:c>
       <x:c r="G19" s="21" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="H19" s="23" t="n">
-        <x:v>0.0005727727874330161</x:v>
+        <x:v>0.0004140736323130022</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2293,21 +2336,67 @@
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="5" t="str">
-        <x:v>Final latency</x:v>
+        <x:v>F01 FP32 288px</x:v>
       </x:c>
       <x:c r="B2" s="6" t="str">
-        <x:v>Chưa có artifact</x:v>
-      </x:c>
-      <x:c r="C2" s="6"/>
-      <x:c r="D2" s="21"/>
+        <x:v>Tesla T4</x:v>
+      </x:c>
+      <x:c r="C2" s="6" t="str">
+        <x:v>FP32</x:v>
+      </x:c>
+      <x:c r="D2" s="21" t="n">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="E2" s="21" t="n">
         <x:v>288</x:v>
       </x:c>
-      <x:c r="F2" s="21"/>
-      <x:c r="G2" s="20"/>
-      <x:c r="H2" s="20"/>
-      <x:c r="I2" s="20"/>
-      <x:c r="J2" s="24"/>
+      <x:c r="F2" s="27" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G2" s="20" t="n">
+        <x:v>31.948846499972205</x:v>
+      </x:c>
+      <x:c r="H2" s="20" t="n">
+        <x:v>49.85229550009079</x:v>
+      </x:c>
+      <x:c r="I2" s="20" t="n">
+        <x:v>57.364511509831566</x:v>
+      </x:c>
+      <x:c r="J2" s="24" t="n">
+        <x:v>31.300034572480417</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" t="str">
+        <x:v>F01 FP32 288px</x:v>
+      </x:c>
+      <x:c r="B3" t="str">
+        <x:v>Tesla T4</x:v>
+      </x:c>
+      <x:c r="C3" t="str">
+        <x:v>FP32</x:v>
+      </x:c>
+      <x:c r="D3" s="29" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="E3" s="29" t="n">
+        <x:v>288</x:v>
+      </x:c>
+      <x:c r="F3" s="28" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G3" s="30" t="n">
+        <x:v>232.14370099981352</x:v>
+      </x:c>
+      <x:c r="H3" s="30" t="n">
+        <x:v>237.94508469998163</x:v>
+      </x:c>
+      <x:c r="I3" s="30" t="n">
+        <x:v>243.31626416999825</x:v>
+      </x:c>
+      <x:c r="J3" s="30" t="n">
+        <x:v>137.84565276671327</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2339,10 +2428,10 @@
         <x:v>Trạng thái</x:v>
       </x:c>
       <x:c r="B2" s="26" t="str">
-        <x:v>Báo cáo tiến độ; final chưa đủ 3 seed</x:v>
+        <x:v>Đã hoàn thành các lượt chạy Colab</x:v>
       </x:c>
       <x:c r="C2" s="7" t="str">
-        <x:v>Chưa hoàn tất</x:v>
+        <x:v>Final đủ 3 seed; có benchmark batch 1/32</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
@@ -2350,10 +2439,10 @@
         <x:v>Số lượt huấn luyện hoàn thành</x:v>
       </x:c>
       <x:c r="B3" s="26" t="n">
-        <x:v>19</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C3" s="7" t="str">
-        <x:v>19 lượt, 190 epoch</x:v>
+        <x:v>20 lượt, 200 epoch</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="24" customHeight="1">
@@ -2402,13 +2491,13 @@
     </x:row>
     <x:row r="8" ht="24" customHeight="1">
       <x:c r="A8" s="5" t="str">
-        <x:v>Macro-F1 test final tạm thời</x:v>
+        <x:v>Macro-F1 test final</x:v>
       </x:c>
       <x:c r="B8" s="26" t="str">
-        <x:v>98.00 ± 0.01%</x:v>
+        <x:v>97.98 ± 0.03%</x:v>
       </x:c>
       <x:c r="C8" s="7" t="str">
-        <x:v>2 seed: 0, 1</x:v>
+        <x:v>3 seed: 0, 1, 2</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="24" customHeight="1">
@@ -2416,10 +2505,10 @@
         <x:v>Cải thiện macro-F1 test (điểm %)</x:v>
       </x:c>
       <x:c r="B9" s="20" t="n">
-        <x:v>0.8779842885065503</x:v>
+        <x:v>0.8584655260462482</x:v>
       </x:c>
       <x:c r="C9" s="7" t="str">
-        <x:v>Tạm thời; số seed khác nhau</x:v>
+        <x:v>Cùng 3 seed: 0, 1, 2</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="24" customHeight="1">
@@ -2427,7 +2516,7 @@
         <x:v>Train + validation ghi trong log (giờ)</x:v>
       </x:c>
       <x:c r="B10" s="20" t="n">
-        <x:v>4.517813500533057</x:v>
+        <x:v>4.770251404556668</x:v>
       </x:c>
       <x:c r="C10" s="7" t="str">
         <x:v>Không gồm setup, inference, sync Drive</x:v>
@@ -2438,21 +2527,32 @@
         <x:v>Checkpoint trên Drive (GiB)</x:v>
       </x:c>
       <x:c r="B11" s="20" t="n">
-        <x:v>11.368872692808509</x:v>
+        <x:v>12.198768958449364</x:v>
       </x:c>
       <x:c r="C11" s="7" t="str">
-        <x:v>best.pt + last.pt; không đưa lên Git</x:v>
+        <x:v>40 file best.pt + last.pt; không đưa lên Git</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="24" customHeight="1">
       <x:c r="A12" s="5" t="str">
-        <x:v>Còn thiếu</x:v>
-      </x:c>
-      <x:c r="B12" s="26" t="str">
-        <x:v>F01 seed2; final latency batch1/32; tên GPU</x:v>
+        <x:v>p95 final batch 1 (ms)</x:v>
+      </x:c>
+      <x:c r="B12" s="20" t="n">
+        <x:v>49.85229550009079</x:v>
       </x:c>
       <x:c r="C12" s="7" t="str">
-        <x:v>Chưa hoàn tất</x:v>
+        <x:v>Tesla T4; chưa gồm đọc/resize ảnh</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" t="str">
+        <x:v>Tự chấm mục I</x:v>
+      </x:c>
+      <x:c r="B13" s="31" t="str">
+        <x:v>18 / 19</x:v>
+      </x:c>
+      <x:c r="C13" t="str">
+        <x:v>I4a chưa chấm; final không dùng TS</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>